<commit_message>
Format Webkey comparable FS Excel for Schedule III presentation
Co-authored-by: shrikant2891 <shrikant2891@gmail.com>
</commit_message>
<xml_diff>
--- a/WEBKEY_SOLUTIONS_FS_FY2025-26_Comparable.xlsx
+++ b/WEBKEY_SOLUTIONS_FS_FY2025-26_Comparable.xlsx
@@ -20,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,17 +33,46 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,13 +80,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,6 +510,13 @@
   </sheetPr>
   <dimension ref="B2:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
@@ -432,365 +526,409 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>CIN: U62099DL2024PTC433481</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Balance Sheet as at 31 March 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>(Amount in ₹ unless otherwise stated)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="1" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Particulars</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>As at 31.03.2026</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>As at 31.03.2025</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Note No.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>As at
+31 March 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>As at
+31 March 2025</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>I. EQUITY AND LIABILITIES</t>
         </is>
       </c>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>(1) Shareholders' funds</t>
         </is>
       </c>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (a) Share capital</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="10" t="n">
         <v>50000</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="10" t="n">
         <v>50000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (b) Reserves and surplus</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="10" t="n">
         <v>-96257.16</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="10" t="n">
         <v>-56679.6</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="1" t="inlineStr"/>
-      <c r="D12" t="n">
+      <c r="B12" s="11" t="inlineStr"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="13" t="n">
         <v>-46257.16</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="13" t="n">
         <v>-6679.6</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>(2) Non-current liabilities</t>
         </is>
       </c>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (a) Long-term borrowings</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="D14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="1" t="inlineStr"/>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="B15" s="11" t="inlineStr"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>(3) Current liabilities</t>
         </is>
       </c>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (a) Short-term borrowings</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="10" t="n">
         <v>45000</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (b) Trade payables</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="9" t="n">
         <v>5</v>
       </c>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        (i) total outstanding dues of micro and small enterprises</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        (i) Total outstanding dues of micro and small enterprises</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        (ii) total outstanding dues of creditors other than MSME</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        (ii) Total outstanding dues of creditors other than MSME</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="10" t="n">
         <v>621146</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (c) Other current liabilities</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="10" t="n">
         <v>51149.91</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (d) Short-term provisions</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="D22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="10" t="n">
         <v>10000</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="1" t="inlineStr"/>
-      <c r="D23" t="n">
+      <c r="B23" s="11" t="inlineStr"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="13" t="n">
         <v>717295.91</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="13" t="n">
         <v>10000</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="13" t="n">
         <v>671038.75</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="13" t="n">
         <v>3320.4</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" s="8" t="inlineStr"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>II. ASSETS</t>
         </is>
       </c>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>(1) Non-current assets</t>
         </is>
       </c>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (a) Property, plant and equipment</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="10" t="n">
         <v>72283.25</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="1" t="inlineStr"/>
-      <c r="D29" t="n">
+      <c r="B29" s="11" t="inlineStr"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="13" t="n">
         <v>72283.25</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>(2) Current assets</t>
         </is>
       </c>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (a) Trade receivables</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="10" t="n">
         <v>77000</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    (b) Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="10" t="n">
         <v>521755.5</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="10" t="n">
         <v>3320.4</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="1" t="inlineStr"/>
-      <c r="D33" t="n">
+      <c r="B33" s="11" t="inlineStr"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="13" t="n">
         <v>598755.5</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="13" t="n">
         <v>3320.4</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="13" t="n">
         <v>671038.75</v>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="13" t="n">
         <v>3320.4</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Check (Total equity and liabilities − Total assets)</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="10" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B4:E4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -803,170 +941,213 @@
   </sheetPr>
   <dimension ref="B2:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>WEBKEY SOLUTIONS PRIVATE LIMITED</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>CIN: U62099DL2024PTC433481</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Statement of Profit and Loss for the year ended 31 March 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>(Amount in ₹)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="1" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Particulars</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>Year ended 31.03.2026</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>Year ended 31.03.2025</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Note No.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Year ended
+31 March 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Year ended
+31 March 2025</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Revenue from operations</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="10" t="n">
         <v>1526001</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="10" t="n">
         <v>330001</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="n">
         <v>1526001</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="13" t="n">
         <v>330001</v>
       </c>
     </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+    </row>
     <row r="11">
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Expenses</t>
         </is>
       </c>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Purchase / project costs</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="10" t="n">
         <v>450000</v>
       </c>
+      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Employee benefit expense</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="10" t="n">
         <v>866188.8</v>
       </c>
+      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Depreciation and amortisation</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="10" t="n">
         <v>3132</v>
       </c>
+      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Other expenses</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="10" t="n">
         <v>246257.66</v>
       </c>
+      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="13" t="n">
         <v>1565578.46</v>
       </c>
+      <c r="E16" s="12" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="inlineStr"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Profit/(loss) before tax</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="13" t="n">
         <v>-39577.46</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="13" t="n">
         <v>-56680</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Profit/(loss) for the year</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="13" t="n">
         <v>-39577.46</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="13" t="n">
         <v>-56680</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B4:E4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -979,259 +1160,267 @@
   </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Ledger</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Map Code</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>31.03.2026 Net (Dr+/Cr-)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>31.03.2025 Net (Dr+/Cr-)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>BS / P&amp;L line</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Share capital (Lokesh + Ritu)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="10" t="n">
         <v>-50000</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="10" t="n">
         <v>-50000</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>BS Share capital</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Profit &amp; Loss A/c (debit b/f)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>RS-OPEN</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="10" t="n">
         <v>56679.7</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="10" t="n">
         <v>56679.7</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Reserves (opening loss)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Unsecured loans</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>STB</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="10" t="n">
         <v>-45000</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>ST borrowings</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Sundry creditors</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>TP-OTH</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="10" t="n">
         <v>-621146</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Trade payables</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Duties &amp; taxes + audit payable</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>OCL</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="10" t="n">
         <v>-51149.91</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="10" t="n">
         <v>-10000</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Other CL / provisions</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>PPE net</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>PPE</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="10" t="n">
         <v>72283.25</v>
       </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>PPE</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Trade receivables</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>TR</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="10" t="n">
         <v>77000</v>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Trade receivables</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Bank</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>CASH</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="10" t="n">
         <v>521755.5</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="10" t="n">
         <v>3320.3</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>IT Services</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>REV</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="10" t="n">
         <v>-1526000</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="10" t="n">
         <v>-330001</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Design &amp; printing</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>COGS</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="10" t="n">
         <v>450000</v>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Purchase</t>
         </is>
@@ -1248,55 +1437,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A8"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Chartered Accountant — review notes (draft)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>1. Figures derived from TrialBaWebkeyl.xlsx (1-Apr-25 to 31-Mar-26).</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2. Prior year comparatives from audited Balance Sheet as at 31.03.2025 (WEBKEY SOLUTIONS PRIVATE LIMITED.xlsx); PY shows minimal operations.</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3. Profit &amp; Loss A/c in Tally is a DEBIT balance (accumulated loss ₹56,679.70) — not a credit profit.</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>2. Prior year comparatives from audited Balance Sheet as at 31.03.2025.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4. Unsecured loans ₹45,000 classified as short-term borrowings; reclassify to long-term if terms exceed 12 months.</t>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>3. Profit &amp; Loss A/c in Tally is a DEBIT balance (accumulated loss ₹56,679.70).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5. MSME trade payable break-up not in TB — disclose when ageing is available.</t>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>4. Unsecured loans ₹45,000 classified as short-term borrowings pending loan agreement review.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6. Income tax: assessability and provisions to be confirmed before final sign-off.</t>
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>5. MSME trade payable break-up to be added when ageing is available.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7. Schedule III notes 1–18 (policies, related party, contingencies, auditor remuneration) to be completed before audit report.</t>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>6. Income tax and full Schedule III notes 1–18 to be completed before audit report and UDIN.</t>
         </is>
       </c>
     </row>
@@ -1311,66 +1503,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B6"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Company name</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>WEBKEY SOLUTIONS PRIVATE LIMITED</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Registered office</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>POLE NO-58, GROUND FLOOR, VILLAGE DHANSA, NEW DELHI, South West Delhi- 110073</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>CIN</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>U62099DL2024PTC433481</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Financial year</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>2025-26 (year ended 31 March 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Auditor</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>G R B &amp; CO</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>FRN</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>040755N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Source TB</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>TrialBaWebkeyl.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Source PY FS</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>WEBKEY SOLUTIONS PRIVATE LIMITED.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>